<commit_message>
Add conductance mapping and refactor model filter
Updated for conductance data and conversion to salinity.
Updated function to keep or remove specified logger relationships.
Moved station mapping to be more useful.
</commit_message>
<xml_diff>
--- a/Water quality/Data/Raw-data/Flow_logger_locations.xlsx
+++ b/Water quality/Data/Raw-data/Flow_logger_locations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Erica.Williams\Documents\GitHub\HSM-and-mapping\Water quality\Data\Raw-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7990421-3CCE-471C-A4D7-EB3E7591E5BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E7F316F-DBBC-4310-8F25-C6997DC2347F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="35">
   <si>
     <t>Site</t>
   </si>
@@ -122,6 +122,9 @@
   </si>
   <si>
     <t>USGS-02310700</t>
+  </si>
+  <si>
+    <t>HO</t>
   </si>
 </sst>
 </file>
@@ -810,7 +813,7 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="B21" t="s">
         <v>27</v>
@@ -929,7 +932,7 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="B28" t="s">
         <v>33</v>
@@ -946,7 +949,7 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="B29" t="s">
         <v>33</v>

</xml_diff>

<commit_message>
Improve flow-salinity modeling and data loading
Added naming to loggers for consistency.
Added code for rain data .
Made load_WQ_data optional for flow/rain. Enhance fit_salinity_flow_models to use station Names, handle zero-flow days, use robust quantile-based start values, and ensure sufficient data checks.
Rewrote ggplot_hyperbolic_fit to support plotting all models (patchwork).
</commit_message>
<xml_diff>
--- a/Water quality/Data/Raw-data/Flow_logger_locations.xlsx
+++ b/Water quality/Data/Raw-data/Flow_logger_locations.xlsx
@@ -1,26 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Erica.Williams\Documents\GitHub\HSM-and-mapping\Water quality\Data\Raw-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E7F316F-DBBC-4310-8F25-C6997DC2347F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{193E05E8-4DDE-4A73-87FF-6E2AEAA502F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="46">
   <si>
     <t>Site</t>
   </si>
@@ -125,13 +138,46 @@
   </si>
   <si>
     <t>HO</t>
+  </si>
+  <si>
+    <t>S49_R</t>
+  </si>
+  <si>
+    <t>Rain</t>
+  </si>
+  <si>
+    <t>S97_R</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>US1</t>
+  </si>
+  <si>
+    <t>A1A</t>
+  </si>
+  <si>
+    <t>S49</t>
+  </si>
+  <si>
+    <t>S80</t>
+  </si>
+  <si>
+    <t>S97</t>
+  </si>
+  <si>
+    <t>USGS-02277110</t>
+  </si>
+  <si>
+    <t>USGS-02277100</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -143,6 +189,12 @@
       <sz val="10"/>
       <color rgb="FF1B1B1B"/>
       <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF334155"/>
+      <name val="Verdana"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -166,9 +218,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -465,13 +518,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E29"/>
-  <sheetFormatPr defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:F33"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -487,8 +540,11 @@
       <c r="E1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -504,8 +560,11 @@
       <c r="E2">
         <v>-83.377499999999998</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -521,8 +580,11 @@
       <c r="E3">
         <v>-83.086667000000006</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -538,8 +600,11 @@
       <c r="E4">
         <v>-82.769001071597003</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -555,8 +620,11 @@
       <c r="E5">
         <v>-83.162099999999995</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -572,8 +640,11 @@
       <c r="E6">
         <v>-83.062749999999994</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -589,8 +660,11 @@
       <c r="E7">
         <v>-83.241699999999994</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>5</v>
       </c>
@@ -606,8 +680,11 @@
       <c r="E8">
         <v>-83.341700000000003</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>5</v>
       </c>
@@ -623,8 +700,11 @@
       <c r="E9">
         <v>-83.022779999999997</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -640,8 +720,11 @@
       <c r="E10">
         <v>-80.288118999999995</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -657,8 +740,11 @@
       <c r="E11">
         <v>-80.258364</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F11" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>16</v>
       </c>
@@ -674,8 +760,11 @@
       <c r="E12">
         <v>-80.207002000000003</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F12" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>16</v>
       </c>
@@ -691,8 +780,11 @@
       <c r="E13">
         <v>-80.359804999999994</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F13" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>16</v>
       </c>
@@ -708,8 +800,11 @@
       <c r="E14">
         <v>-80.285263</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F14" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>16</v>
       </c>
@@ -725,8 +820,11 @@
       <c r="E15">
         <v>-80.34066</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F15" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>23</v>
       </c>
@@ -742,8 +840,11 @@
       <c r="E16" s="1">
         <v>-82.769001071597003</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>23</v>
       </c>
@@ -759,8 +860,11 @@
       <c r="E17" s="1">
         <v>-82.769001071597003</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F17" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>23</v>
       </c>
@@ -776,8 +880,11 @@
       <c r="E18">
         <v>-82.765833008482403</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F18" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>23</v>
       </c>
@@ -793,8 +900,11 @@
       <c r="E19">
         <v>-82.747638888888801</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F19" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>23</v>
       </c>
@@ -810,8 +920,11 @@
       <c r="E20">
         <v>-82.690638888888898</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F20" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>34</v>
       </c>
@@ -827,8 +940,11 @@
       <c r="E21">
         <v>-82.695706281747107</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F21" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>23</v>
       </c>
@@ -844,8 +960,11 @@
       <c r="E22">
         <v>-82.732891666666603</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F22" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>23</v>
       </c>
@@ -861,8 +980,11 @@
       <c r="E23">
         <v>-82.645805555555498</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F23" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>23</v>
       </c>
@@ -878,8 +1000,11 @@
       <c r="E24">
         <v>-82.637881756271497</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F24" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>23</v>
       </c>
@@ -895,8 +1020,11 @@
       <c r="E25">
         <v>-82.635188270857199</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F25" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>23</v>
       </c>
@@ -912,8 +1040,11 @@
       <c r="E26">
         <v>-82.635188270857199</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F26" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>23</v>
       </c>
@@ -929,8 +1060,11 @@
       <c r="E27">
         <v>-82.616769865935098</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F27" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>34</v>
       </c>
@@ -946,8 +1080,11 @@
       <c r="E28">
         <v>-82.617926267019001</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F28" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>34</v>
       </c>
@@ -962,6 +1099,89 @@
       </c>
       <c r="E29">
         <v>-82.617926267019001</v>
+      </c>
+      <c r="F29" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>16</v>
+      </c>
+      <c r="B30" t="s">
+        <v>35</v>
+      </c>
+      <c r="C30" t="s">
+        <v>36</v>
+      </c>
+      <c r="D30" s="2">
+        <v>27.261139</v>
+      </c>
+      <c r="E30" s="2">
+        <v>-80.359397000000001</v>
+      </c>
+      <c r="F30" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>16</v>
+      </c>
+      <c r="B31" t="s">
+        <v>37</v>
+      </c>
+      <c r="C31" t="s">
+        <v>36</v>
+      </c>
+      <c r="D31">
+        <v>27.205774999999999</v>
+      </c>
+      <c r="E31">
+        <v>-80.340772000000001</v>
+      </c>
+      <c r="F31" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>16</v>
+      </c>
+      <c r="B32" t="s">
+        <v>44</v>
+      </c>
+      <c r="C32" t="s">
+        <v>11</v>
+      </c>
+      <c r="D32">
+        <v>27.199384999999999</v>
+      </c>
+      <c r="E32">
+        <v>-80.207002000000003</v>
+      </c>
+      <c r="F32" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>16</v>
+      </c>
+      <c r="B33" t="s">
+        <v>45</v>
+      </c>
+      <c r="C33" t="s">
+        <v>11</v>
+      </c>
+      <c r="D33">
+        <v>27.201958000000001</v>
+      </c>
+      <c r="E33">
+        <v>-80.258364</v>
+      </c>
+      <c r="F33" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Switch site to WI; update WQ/HSM pipelines
WI model progress
Added CSI install code
Highlighted WI/Flow loggers in maps
Tweak output plot settings: lower DPI, change compression, and rasterize DPI.
In WQ_functions_flow, add informative load messages, drop NA before clustering, print location counts and estimated dist-matrix size, compute haversine distances, and ensure adjacency matrix is symmetric before graph creation.
</commit_message>
<xml_diff>
--- a/Water quality/Data/Raw-data/Flow_logger_locations.xlsx
+++ b/Water quality/Data/Raw-data/Flow_logger_locations.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
   <si>
     <t xml:space="preserve">Site</t>
   </si>
@@ -117,6 +117,24 @@
   </si>
   <si>
     <t xml:space="preserve">USGS-02310700</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WISal1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WISal2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WISal3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WISal4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WISal5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WISal6</t>
   </si>
 </sst>
 </file>
@@ -938,6 +956,108 @@
         <v>-82.617926267019</v>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="s">
+        <v>23</v>
+      </c>
+      <c r="B30" t="s">
+        <v>35</v>
+      </c>
+      <c r="C30" t="s">
+        <v>11</v>
+      </c>
+      <c r="D30" t="n">
+        <v>28.90296</v>
+      </c>
+      <c r="E30" t="n">
+        <v>-82.64148</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="s">
+        <v>23</v>
+      </c>
+      <c r="B31" t="s">
+        <v>36</v>
+      </c>
+      <c r="C31" t="s">
+        <v>11</v>
+      </c>
+      <c r="D31" t="n">
+        <v>29.00113</v>
+      </c>
+      <c r="E31" t="n">
+        <v>-82.76583</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s">
+        <v>23</v>
+      </c>
+      <c r="B32" t="s">
+        <v>37</v>
+      </c>
+      <c r="C32" t="s">
+        <v>11</v>
+      </c>
+      <c r="D32" t="n">
+        <v>29.20413</v>
+      </c>
+      <c r="E32" t="n">
+        <v>-82.769</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s">
+        <v>23</v>
+      </c>
+      <c r="B33" t="s">
+        <v>38</v>
+      </c>
+      <c r="C33" t="s">
+        <v>11</v>
+      </c>
+      <c r="D33" t="n">
+        <v>28.92528</v>
+      </c>
+      <c r="E33" t="n">
+        <v>-82.69064</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s">
+        <v>23</v>
+      </c>
+      <c r="B34" t="s">
+        <v>39</v>
+      </c>
+      <c r="C34" t="s">
+        <v>11</v>
+      </c>
+      <c r="D34" t="n">
+        <v>28.91169</v>
+      </c>
+      <c r="E34" t="n">
+        <v>-82.74764</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="s">
+        <v>23</v>
+      </c>
+      <c r="B35" t="s">
+        <v>40</v>
+      </c>
+      <c r="C35" t="s">
+        <v>11</v>
+      </c>
+      <c r="D35" t="n">
+        <v>28.75158</v>
+      </c>
+      <c r="E35" t="n">
+        <v>-82.73289</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>